<commit_message>
Fix portfolio underlying asset display
</commit_message>
<xml_diff>
--- a/backend/data/transactions.xlsx
+++ b/backend/data/transactions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PWMS\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DB78E99-BCBA-4EA2-A588-05FE947D15A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A57CDCA7-1DE4-41F0-9CC7-D1B8A97D9AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="2" xr2:uid="{EF3E2500-DA9F-4B00-9FD1-12C576E189BD}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4879" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4846" uniqueCount="240">
   <si>
     <t>Family Name</t>
   </si>
@@ -764,6 +764,9 @@
   <si>
     <t>Tata Power</t>
   </si>
+  <si>
+    <t>IE000QX7EHP1</t>
+  </si>
 </sst>
 </file>
 
@@ -900,7 +903,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -924,7 +927,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
@@ -6339,7 +6341,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10DD8D7D-9FD3-4B34-BD1A-D08D200D033F}">
-  <dimension ref="A1:L520"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:L519"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" customWidth="1"/>
@@ -6393,7 +6396,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
@@ -6432,7 +6435,7 @@
         <v>390323.79</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>10</v>
       </c>
@@ -6471,7 +6474,7 @@
         <v>408076.19</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>10</v>
       </c>
@@ -6509,7 +6512,7 @@
         <v>132400.78</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>10</v>
       </c>
@@ -6547,7 +6550,7 @@
         <v>295791.01</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
@@ -6586,7 +6589,7 @@
         <v>67047.289999999994</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
@@ -6625,7 +6628,7 @@
         <v>176723.68</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>10</v>
       </c>
@@ -6663,7 +6666,7 @@
         <v>240876.26</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
@@ -6702,7 +6705,7 @@
         <v>381277.46</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
         <v>10</v>
       </c>
@@ -6741,7 +6744,7 @@
         <v>24126.79</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>10</v>
       </c>
@@ -6779,7 +6782,7 @@
         <v>447388.04</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
         <v>10</v>
       </c>
@@ -6817,7 +6820,7 @@
         <v>144346.53</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
         <v>10</v>
       </c>
@@ -6855,7 +6858,7 @@
         <v>196696.05</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
         <v>10</v>
       </c>
@@ -6894,7 +6897,7 @@
         <v>256261.48</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>10</v>
       </c>
@@ -6933,7 +6936,7 @@
         <v>107318.18</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>10</v>
       </c>
@@ -6972,7 +6975,7 @@
         <v>41562.19</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
         <v>10</v>
       </c>
@@ -7011,7 +7014,7 @@
         <v>318898.55</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
         <v>10</v>
       </c>
@@ -7050,7 +7053,7 @@
         <v>173169.76</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
         <v>10</v>
       </c>
@@ -7089,7 +7092,7 @@
         <v>395357.92</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
         <v>10</v>
       </c>
@@ -7128,7 +7131,7 @@
         <v>9349.24</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
         <v>10</v>
       </c>
@@ -7166,7 +7169,7 @@
         <v>6616.99</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
         <v>10</v>
       </c>
@@ -7205,7 +7208,7 @@
         <v>16180.22</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
         <v>10</v>
       </c>
@@ -7244,7 +7247,7 @@
         <v>19219.41</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
         <v>10</v>
       </c>
@@ -7283,7 +7286,7 @@
         <v>25246.43</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
         <v>10</v>
       </c>
@@ -7322,7 +7325,7 @@
         <v>47243.82</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
         <v>10</v>
       </c>
@@ -7361,7 +7364,7 @@
         <v>29983.360000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
         <v>10</v>
       </c>
@@ -7400,7 +7403,7 @@
         <v>14418.05</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="s">
         <v>10</v>
       </c>
@@ -7439,7 +7442,7 @@
         <v>17510.37</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
         <v>10</v>
       </c>
@@ -7478,7 +7481,7 @@
         <v>184383.25</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
         <v>10</v>
       </c>
@@ -7517,7 +7520,7 @@
         <v>11709.17</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
         <v>10</v>
       </c>
@@ -7556,7 +7559,7 @@
         <v>402579.83</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="6" t="s">
         <v>10</v>
       </c>
@@ -7594,7 +7597,7 @@
         <v>184102.46</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
         <v>10</v>
       </c>
@@ -7633,7 +7636,7 @@
         <v>295804.09999999998</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="6" t="s">
         <v>10</v>
       </c>
@@ -7671,7 +7674,7 @@
         <v>576097.03</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
         <v>10</v>
       </c>
@@ -7710,7 +7713,7 @@
         <v>195392.73</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="6" t="s">
         <v>10</v>
       </c>
@@ -7749,7 +7752,7 @@
         <v>20141.509999999998</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
         <v>10</v>
       </c>
@@ -7787,7 +7790,7 @@
         <v>106069.83</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="6" t="s">
         <v>10</v>
       </c>
@@ -7826,7 +7829,7 @@
         <v>2912.17</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
         <v>10</v>
       </c>
@@ -7864,7 +7867,7 @@
         <v>224489.29</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="6" t="s">
         <v>10</v>
       </c>
@@ -7903,7 +7906,7 @@
         <v>4858.07</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="6" t="s">
         <v>10</v>
       </c>
@@ -7942,7 +7945,7 @@
         <v>313823.71999999997</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
         <v>10</v>
       </c>
@@ -7981,7 +7984,7 @@
         <v>67781.63</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
         <v>10</v>
       </c>
@@ -8020,7 +8023,7 @@
         <v>2247.73</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="6" t="s">
         <v>10</v>
       </c>
@@ -8058,7 +8061,7 @@
         <v>14712.04</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6" t="s">
         <v>10</v>
       </c>
@@ -8097,7 +8100,7 @@
         <v>194831.2</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="6" t="s">
         <v>10</v>
       </c>
@@ -8136,7 +8139,7 @@
         <v>44800.11</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="6" t="s">
         <v>10</v>
       </c>
@@ -8175,7 +8178,7 @@
         <v>30305.02</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="6" t="s">
         <v>10</v>
       </c>
@@ -8214,7 +8217,7 @@
         <v>573352.52</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="6" t="s">
         <v>10</v>
       </c>
@@ -8252,7 +8255,7 @@
         <v>106686.13</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="6" t="s">
         <v>10</v>
       </c>
@@ -8291,7 +8294,7 @@
         <v>303983.98</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="6" t="s">
         <v>10</v>
       </c>
@@ -8329,7 +8332,7 @@
         <v>38533.4</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="6" t="s">
         <v>10</v>
       </c>
@@ -8367,7 +8370,7 @@
         <v>58934.37</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="6" t="s">
         <v>10</v>
       </c>
@@ -8405,7 +8408,7 @@
         <v>654651.81000000006</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="6" t="s">
         <v>10</v>
       </c>
@@ -8444,7 +8447,7 @@
         <v>560659.81999999995</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="6" t="s">
         <v>10</v>
       </c>
@@ -8482,7 +8485,7 @@
         <v>408193.47</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="6" t="s">
         <v>10</v>
       </c>
@@ -8521,7 +8524,7 @@
         <v>802045.65</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
         <v>10</v>
       </c>
@@ -8560,7 +8563,7 @@
         <v>109916.02</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="6" t="s">
         <v>10</v>
       </c>
@@ -8599,7 +8602,7 @@
         <v>33120.67</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="6" t="s">
         <v>10</v>
       </c>
@@ -8637,7 +8640,7 @@
         <v>276404.32</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="6" t="s">
         <v>10</v>
       </c>
@@ -8676,7 +8679,7 @@
         <v>10061.18</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="6" t="s">
         <v>10</v>
       </c>
@@ -8715,7 +8718,7 @@
         <v>58008.36</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="6" t="s">
         <v>10</v>
       </c>
@@ -8753,7 +8756,7 @@
         <v>78419.64</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="6" t="s">
         <v>10</v>
       </c>
@@ -8791,7 +8794,7 @@
         <v>166902.28</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="6" t="s">
         <v>10</v>
       </c>
@@ -8830,7 +8833,7 @@
         <v>3758.28</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="6" t="s">
         <v>10</v>
       </c>
@@ -8869,7 +8872,7 @@
         <v>115676.51</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="6" t="s">
         <v>10</v>
       </c>
@@ -8908,7 +8911,7 @@
         <v>7935.47</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="6" t="s">
         <v>10</v>
       </c>
@@ -8947,7 +8950,7 @@
         <v>7912.85</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="6" t="s">
         <v>10</v>
       </c>
@@ -8986,7 +8989,7 @@
         <v>4898.9799999999996</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="6" t="s">
         <v>10</v>
       </c>
@@ -9025,7 +9028,7 @@
         <v>565956.71</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="6" t="s">
         <v>10</v>
       </c>
@@ -9063,7 +9066,7 @@
         <v>12612.85</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="6" t="s">
         <v>10</v>
       </c>
@@ -9102,7 +9105,7 @@
         <v>2034.55</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="6" t="s">
         <v>10</v>
       </c>
@@ -9141,7 +9144,7 @@
         <v>16740.41</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="6" t="s">
         <v>10</v>
       </c>
@@ -9180,7 +9183,7 @@
         <v>5336.35</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="6" t="s">
         <v>10</v>
       </c>
@@ -9218,7 +9221,7 @@
         <v>11424.55</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="6" t="s">
         <v>10</v>
       </c>
@@ -9257,7 +9260,7 @@
         <v>16711.68</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="6" t="s">
         <v>10</v>
       </c>
@@ -9296,7 +9299,7 @@
         <v>80354.69</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="6" t="s">
         <v>10</v>
       </c>
@@ -9334,7 +9337,7 @@
         <v>109762.97</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="6" t="s">
         <v>10</v>
       </c>
@@ -9372,7 +9375,7 @@
         <v>327722.2</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="6" t="s">
         <v>10</v>
       </c>
@@ -9411,7 +9414,7 @@
         <v>161264.68</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="6" t="s">
         <v>10</v>
       </c>
@@ -9450,7 +9453,7 @@
         <v>15578.41</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="6" t="s">
         <v>10</v>
       </c>
@@ -9489,7 +9492,7 @@
         <v>56781.23</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="6" t="s">
         <v>10</v>
       </c>
@@ -9527,7 +9530,7 @@
         <v>15995.42</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="6" t="s">
         <v>10</v>
       </c>
@@ -9566,7 +9569,7 @@
         <v>9559.81</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="6" t="s">
         <v>10</v>
       </c>
@@ -9604,7 +9607,7 @@
         <v>22598.28</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="6" t="s">
         <v>10</v>
       </c>
@@ -9643,7 +9646,7 @@
         <v>44947.62</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="6" t="s">
         <v>10</v>
       </c>
@@ -9682,7 +9685,7 @@
         <v>20184.43</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="6" t="s">
         <v>10</v>
       </c>
@@ -9721,7 +9724,7 @@
         <v>68189.56</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="6" t="s">
         <v>10</v>
       </c>
@@ -9760,7 +9763,7 @@
         <v>80018.87</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="6" t="s">
         <v>10</v>
       </c>
@@ -9799,7 +9802,7 @@
         <v>63414.84</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="6" t="s">
         <v>10</v>
       </c>
@@ -9838,7 +9841,7 @@
         <v>86985.75</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="6" t="s">
         <v>10</v>
       </c>
@@ -9877,7 +9880,7 @@
         <v>23544.28</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="6" t="s">
         <v>10</v>
       </c>
@@ -9916,7 +9919,7 @@
         <v>21885.9</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="6" t="s">
         <v>10</v>
       </c>
@@ -9955,7 +9958,7 @@
         <v>111126.14</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="6" t="s">
         <v>10</v>
       </c>
@@ -9994,7 +9997,7 @@
         <v>4330.16</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="6" t="s">
         <v>10</v>
       </c>
@@ -10033,7 +10036,7 @@
         <v>80430.47</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="6" t="s">
         <v>10</v>
       </c>
@@ -10071,7 +10074,7 @@
         <v>163391.5</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="6" t="s">
         <v>10</v>
       </c>
@@ -10109,7 +10112,7 @@
         <v>4590.3500000000004</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="6" t="s">
         <v>10</v>
       </c>
@@ -10148,7 +10151,7 @@
         <v>14622.63</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="6" t="s">
         <v>10</v>
       </c>
@@ -10187,7 +10190,7 @@
         <v>7301.06</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="6" t="s">
         <v>10</v>
       </c>
@@ -10225,7 +10228,7 @@
         <v>43639.54</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="6" t="s">
         <v>10</v>
       </c>
@@ -10264,7 +10267,7 @@
         <v>164401.54</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="6" t="s">
         <v>10</v>
       </c>
@@ -10303,7 +10306,7 @@
         <v>222139.32</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="6" t="s">
         <v>10</v>
       </c>
@@ -10342,7 +10345,7 @@
         <v>167661.41</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="6" t="s">
         <v>10</v>
       </c>
@@ -10381,7 +10384,7 @@
         <v>40749.370000000003</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="6" t="s">
         <v>10</v>
       </c>
@@ -10419,7 +10422,7 @@
         <v>100452.56</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="6" t="s">
         <v>10</v>
       </c>
@@ -10458,7 +10461,7 @@
         <v>110491.74</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="6" t="s">
         <v>10</v>
       </c>
@@ -10497,7 +10500,7 @@
         <v>57496.91</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="6" t="s">
         <v>10</v>
       </c>
@@ -10536,7 +10539,7 @@
         <v>147039.69</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="6" t="s">
         <v>10</v>
       </c>
@@ -10575,7 +10578,7 @@
         <v>110036.74</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="6" t="s">
         <v>10</v>
       </c>
@@ -10614,7 +10617,7 @@
         <v>557109.11</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="6" t="s">
         <v>10</v>
       </c>
@@ -10652,7 +10655,7 @@
         <v>199768.28</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="6" t="s">
         <v>10</v>
       </c>
@@ -10691,7 +10694,7 @@
         <v>149243.17000000001</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="6" t="s">
         <v>10</v>
       </c>
@@ -10730,7 +10733,7 @@
         <v>95270.54</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="6" t="s">
         <v>10</v>
       </c>
@@ -10769,7 +10772,7 @@
         <v>196812.34</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="6" t="s">
         <v>10</v>
       </c>
@@ -10808,7 +10811,7 @@
         <v>147837.64000000001</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="6" t="s">
         <v>10</v>
       </c>
@@ -10847,7 +10850,7 @@
         <v>196245.58</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="6" t="s">
         <v>10</v>
       </c>
@@ -10886,7 +10889,7 @@
         <v>198450.61</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="6" t="s">
         <v>10</v>
       </c>
@@ -10925,7 +10928,7 @@
         <v>196134.62</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="6" t="s">
         <v>10</v>
       </c>
@@ -10963,7 +10966,7 @@
         <v>433256.78</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="6" t="s">
         <v>10</v>
       </c>
@@ -11002,7 +11005,7 @@
         <v>273866.34000000003</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="6" t="s">
         <v>10</v>
       </c>
@@ -11041,7 +11044,7 @@
         <v>2031691.23</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="6" t="s">
         <v>10</v>
       </c>
@@ -11080,7 +11083,7 @@
         <v>606656.38</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="6" t="s">
         <v>10</v>
       </c>
@@ -11119,7 +11122,7 @@
         <v>1446751.19</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="6" t="s">
         <v>10</v>
       </c>
@@ -11158,7 +11161,7 @@
         <v>402515.49</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="6" t="s">
         <v>10</v>
       </c>
@@ -11197,7 +11200,7 @@
         <v>789914.42</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="6" t="s">
         <v>10</v>
       </c>
@@ -11236,7 +11239,7 @@
         <v>803732.68</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="6" t="s">
         <v>10</v>
       </c>
@@ -11275,7 +11278,7 @@
         <v>178185.79</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="6" t="s">
         <v>10</v>
       </c>
@@ -11313,7 +11316,7 @@
         <v>589960.4</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="6" t="s">
         <v>10</v>
       </c>
@@ -11351,7 +11354,7 @@
         <v>747002.19</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="6" t="s">
         <v>10</v>
       </c>
@@ -11390,7 +11393,7 @@
         <v>794551.02</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="6" t="s">
         <v>10</v>
       </c>
@@ -11429,7 +11432,7 @@
         <v>708449.27</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="6" t="s">
         <v>10</v>
       </c>
@@ -11468,7 +11471,7 @@
         <v>258877.45</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="6" t="s">
         <v>10</v>
       </c>
@@ -11506,7 +11509,7 @@
         <v>714800.09</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="6" t="s">
         <v>10</v>
       </c>
@@ -11544,7 +11547,7 @@
         <v>4997214.13</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="6" t="s">
         <v>10</v>
       </c>
@@ -11582,7 +11585,7 @@
         <v>7513088.4500000002</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="6" t="s">
         <v>10</v>
       </c>
@@ -11620,7 +11623,7 @@
         <v>2163840.3766999999</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="6" t="s">
         <v>10</v>
       </c>
@@ -11658,7 +11661,7 @@
         <v>2164349.2232999997</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="6" t="s">
         <v>10</v>
       </c>
@@ -11696,7 +11699,7 @@
         <v>2506229.6800000002</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="6" t="s">
         <v>10</v>
       </c>
@@ -11734,7 +11737,7 @@
         <v>2505469.11</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="6" t="s">
         <v>10</v>
       </c>
@@ -11772,7 +11775,7 @@
         <v>426930</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="6" t="s">
         <v>10</v>
       </c>
@@ -11810,7 +11813,7 @@
         <v>5006639.07</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" s="6" t="s">
         <v>10</v>
       </c>
@@ -11848,7 +11851,7 @@
         <v>5014204.72</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" s="6" t="s">
         <v>10</v>
       </c>
@@ -11886,7 +11889,7 @@
         <v>154.28</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" s="6" t="s">
         <v>10</v>
       </c>
@@ -11924,7 +11927,7 @@
         <v>5005813.2</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="6" t="s">
         <v>10</v>
       </c>
@@ -11962,7 +11965,7 @@
         <v>5520107.2400000002</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="6" t="s">
         <v>10</v>
       </c>
@@ -12000,7 +12003,7 @@
         <v>337998.42330000002</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" s="6" t="s">
         <v>10</v>
       </c>
@@ -12038,7 +12041,7 @@
         <v>338077.90669999999</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="6" t="s">
         <v>10</v>
       </c>
@@ -12074,7 +12077,7 @@
         <v>70000000</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="6" t="s">
         <v>10</v>
       </c>
@@ -12110,7 +12113,7 @@
         <v>15600000</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="6" t="s">
         <v>10</v>
       </c>
@@ -12146,7 +12149,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" s="6" t="s">
         <v>10</v>
       </c>
@@ -12182,7 +12185,7 @@
         <v>8001143.96</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" s="6" t="s">
         <v>10</v>
       </c>
@@ -12218,7 +12221,7 @@
         <v>55002277.579999998</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" s="6" t="s">
         <v>10</v>
       </c>
@@ -12254,7 +12257,7 @@
         <v>40000000</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" s="6" t="s">
         <v>10</v>
       </c>
@@ -12290,7 +12293,7 @@
         <v>6001769.8600000003</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" s="6" t="s">
         <v>10</v>
       </c>
@@ -12326,7 +12329,7 @@
         <v>5001470.46</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" s="6" t="s">
         <v>10</v>
       </c>
@@ -12362,7 +12365,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" s="6" t="s">
         <v>10</v>
       </c>
@@ -12398,7 +12401,7 @@
         <v>90666.55</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="6" t="s">
         <v>10</v>
       </c>
@@ -12434,7 +12437,7 @@
         <v>10000000</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="6" t="s">
         <v>10</v>
       </c>
@@ -12559,9 +12562,7 @@
       <c r="D162" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="E162" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E162" s="7"/>
       <c r="F162" s="7" t="s">
         <v>185</v>
       </c>
@@ -12597,9 +12598,7 @@
       <c r="D163" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E163" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E163" s="7"/>
       <c r="F163" s="7" t="s">
         <v>187</v>
       </c>
@@ -12635,9 +12634,7 @@
       <c r="D164" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="E164" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E164" s="7"/>
       <c r="F164" s="7" t="s">
         <v>187</v>
       </c>
@@ -12660,7 +12657,7 @@
         <v>9584000</v>
       </c>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" s="6" t="s">
         <v>10</v>
       </c>
@@ -12673,9 +12670,7 @@
       <c r="D165" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E165" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E165" s="7"/>
       <c r="F165" s="7" t="s">
         <v>185</v>
       </c>
@@ -12696,7 +12691,7 @@
         <v>10500000</v>
       </c>
     </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" s="6" t="s">
         <v>10</v>
       </c>
@@ -12709,9 +12704,7 @@
       <c r="D166" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E166" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E166" s="7"/>
       <c r="F166" s="7" t="s">
         <v>185</v>
       </c>
@@ -12732,7 +12725,7 @@
         <v>2100000</v>
       </c>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" s="6" t="s">
         <v>10</v>
       </c>
@@ -12745,9 +12738,7 @@
       <c r="D167" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E167" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E167" s="7"/>
       <c r="F167" s="7" t="s">
         <v>185</v>
       </c>
@@ -12781,9 +12772,7 @@
       <c r="D168" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="E168" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E168" s="7"/>
       <c r="F168" s="7" t="s">
         <v>186</v>
       </c>
@@ -12804,7 +12793,7 @@
         <v>10033040</v>
       </c>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" s="6" t="s">
         <v>10</v>
       </c>
@@ -12817,13 +12806,13 @@
       <c r="D169" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="E169" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E169" s="7"/>
       <c r="F169" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="G169" s="7"/>
+      <c r="G169" s="7" t="s">
+        <v>239</v>
+      </c>
       <c r="H169" s="8">
         <v>46044</v>
       </c>
@@ -12842,7 +12831,7 @@
         <v>13735506.530772397</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" s="6" t="s">
         <v>10</v>
       </c>
@@ -12855,13 +12844,13 @@
       <c r="D170" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="E170" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E170" s="7"/>
       <c r="F170" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="G170" s="7"/>
+      <c r="G170" s="7" t="s">
+        <v>239</v>
+      </c>
       <c r="H170" s="8">
         <v>46077</v>
       </c>
@@ -12880,7 +12869,7 @@
         <v>4509410.8771436401</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" s="6" t="s">
         <v>116</v>
       </c>
@@ -12893,15 +12882,13 @@
       <c r="D171" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E171" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E171" s="7"/>
       <c r="F171" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G171" s="7" t="str">
+      <c r="G171" s="7" t="e">
         <f>+VLOOKUP(E171,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H171" s="8">
         <v>46240</v>
@@ -12919,7 +12906,7 @@
         <v>938716.26</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" s="6" t="s">
         <v>116</v>
       </c>
@@ -12932,9 +12919,7 @@
       <c r="D172" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E172" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E172" s="7"/>
       <c r="F172" s="6" t="s">
         <v>185</v>
       </c>
@@ -12957,7 +12942,7 @@
         <v>1439969.49</v>
       </c>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" s="6" t="s">
         <v>116</v>
       </c>
@@ -12970,15 +12955,13 @@
       <c r="D173" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E173" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E173" s="7"/>
       <c r="F173" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G173" s="7" t="str">
+      <c r="G173" s="7" t="e">
         <f>+VLOOKUP(E173,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H173" s="8">
         <v>46227</v>
@@ -12996,7 +12979,7 @@
         <v>1153091.93</v>
       </c>
     </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" s="6" t="s">
         <v>116</v>
       </c>
@@ -13009,15 +12992,13 @@
       <c r="D174" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E174" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E174" s="7"/>
       <c r="F174" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G174" s="7" t="str">
+      <c r="G174" s="7" t="e">
         <f>+VLOOKUP(E174,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H174" s="8">
         <v>46225</v>
@@ -13035,7 +13016,7 @@
         <v>242944.3</v>
       </c>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" s="6" t="s">
         <v>116</v>
       </c>
@@ -13048,15 +13029,13 @@
       <c r="D175" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E175" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E175" s="7"/>
       <c r="F175" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G175" s="7" t="str">
+      <c r="G175" s="7" t="e">
         <f>+VLOOKUP(E175,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H175" s="8">
         <v>46224</v>
@@ -13074,7 +13053,7 @@
         <v>1074047.5</v>
       </c>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" s="6" t="s">
         <v>116</v>
       </c>
@@ -13087,15 +13066,13 @@
       <c r="D176" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E176" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E176" s="7"/>
       <c r="F176" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G176" s="7" t="str">
+      <c r="G176" s="7" t="e">
         <f>+VLOOKUP(E176,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H176" s="8">
         <v>46224</v>
@@ -13113,7 +13090,7 @@
         <v>963064.54</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" s="6" t="s">
         <v>116</v>
       </c>
@@ -13126,9 +13103,7 @@
       <c r="D177" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E177" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E177" s="7"/>
       <c r="F177" s="6" t="s">
         <v>185</v>
       </c>
@@ -13151,7 +13126,7 @@
         <v>1793154.61</v>
       </c>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" s="6" t="s">
         <v>116</v>
       </c>
@@ -13164,15 +13139,13 @@
       <c r="D178" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E178" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E178" s="7"/>
       <c r="F178" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G178" s="7" t="str">
+      <c r="G178" s="7" t="e">
         <f>+VLOOKUP(E178,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H178" s="8">
         <v>46217</v>
@@ -13190,7 +13163,7 @@
         <v>287469.78999999998</v>
       </c>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" s="6" t="s">
         <v>116</v>
       </c>
@@ -13203,15 +13176,13 @@
       <c r="D179" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E179" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E179" s="7"/>
       <c r="F179" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G179" s="7" t="str">
+      <c r="G179" s="7" t="e">
         <f>+VLOOKUP(E179,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H179" s="8">
         <v>46211</v>
@@ -13229,7 +13200,7 @@
         <v>1600527.44</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" s="6" t="s">
         <v>116</v>
       </c>
@@ -13242,15 +13213,13 @@
       <c r="D180" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E180" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E180" s="7"/>
       <c r="F180" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G180" s="7" t="str">
+      <c r="G180" s="7" t="e">
         <f>+VLOOKUP(E180,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H180" s="8">
         <v>46210</v>
@@ -13268,7 +13237,7 @@
         <v>730443.9</v>
       </c>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="6" t="s">
         <v>116</v>
       </c>
@@ -13281,15 +13250,13 @@
       <c r="D181" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E181" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E181" s="7"/>
       <c r="F181" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G181" s="7" t="str">
+      <c r="G181" s="7" t="e">
         <f>+VLOOKUP(E181,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H181" s="8">
         <v>46205</v>
@@ -13307,7 +13274,7 @@
         <v>379563.81</v>
       </c>
     </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" s="6" t="s">
         <v>116</v>
       </c>
@@ -13320,9 +13287,7 @@
       <c r="D182" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E182" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E182" s="7"/>
       <c r="F182" s="6" t="s">
         <v>185</v>
       </c>
@@ -13345,7 +13310,7 @@
         <v>496588.13</v>
       </c>
     </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" s="6" t="s">
         <v>116</v>
       </c>
@@ -13358,15 +13323,13 @@
       <c r="D183" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E183" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E183" s="7"/>
       <c r="F183" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G183" s="7" t="str">
+      <c r="G183" s="7" t="e">
         <f>+VLOOKUP(E183,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H183" s="8">
         <v>46197</v>
@@ -13384,7 +13347,7 @@
         <v>1121849.4099999999</v>
       </c>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" s="6" t="s">
         <v>116</v>
       </c>
@@ -13397,9 +13360,7 @@
       <c r="D184" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E184" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E184" s="7"/>
       <c r="F184" s="6" t="s">
         <v>185</v>
       </c>
@@ -13422,7 +13383,7 @@
         <v>2175065.65</v>
       </c>
     </row>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" s="6" t="s">
         <v>116</v>
       </c>
@@ -13435,15 +13396,13 @@
       <c r="D185" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E185" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E185" s="7"/>
       <c r="F185" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G185" s="7" t="str">
+      <c r="G185" s="7" t="e">
         <f>+VLOOKUP(E185,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H185" s="8">
         <v>46182</v>
@@ -13461,7 +13420,7 @@
         <v>1650780.27</v>
       </c>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" s="6" t="s">
         <v>116</v>
       </c>
@@ -13474,9 +13433,7 @@
       <c r="D186" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E186" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E186" s="7"/>
       <c r="F186" s="6" t="s">
         <v>185</v>
       </c>
@@ -13499,7 +13456,7 @@
         <v>1682226.09</v>
       </c>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" s="6" t="s">
         <v>116</v>
       </c>
@@ -13512,15 +13469,13 @@
       <c r="D187" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E187" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E187" s="7"/>
       <c r="F187" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G187" s="7" t="str">
+      <c r="G187" s="7" t="e">
         <f>+VLOOKUP(E187,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H187" s="8">
         <v>46177</v>
@@ -13538,7 +13493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" s="6" t="s">
         <v>116</v>
       </c>
@@ -13551,15 +13506,13 @@
       <c r="D188" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E188" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E188" s="7"/>
       <c r="F188" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G188" s="7" t="str">
+      <c r="G188" s="7" t="e">
         <f>+VLOOKUP(E188,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H188" s="8">
         <v>46175</v>
@@ -13577,7 +13530,7 @@
         <v>217329.66</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" s="6" t="s">
         <v>116</v>
       </c>
@@ -13590,15 +13543,13 @@
       <c r="D189" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E189" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E189" s="7"/>
       <c r="F189" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G189" s="7" t="str">
+      <c r="G189" s="7" t="e">
         <f>+VLOOKUP(E189,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H189" s="8">
         <v>46175</v>
@@ -13616,7 +13567,7 @@
         <v>311689.71999999997</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" s="6" t="s">
         <v>116</v>
       </c>
@@ -13629,9 +13580,7 @@
       <c r="D190" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E190" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E190" s="7"/>
       <c r="F190" s="6" t="s">
         <v>185</v>
       </c>
@@ -13654,7 +13603,7 @@
         <v>79752.800000000003</v>
       </c>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" s="6" t="s">
         <v>116</v>
       </c>
@@ -13667,9 +13616,7 @@
       <c r="D191" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E191" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E191" s="7"/>
       <c r="F191" s="6" t="s">
         <v>185</v>
       </c>
@@ -13692,7 +13639,7 @@
         <v>2130755.84</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" s="6" t="s">
         <v>116</v>
       </c>
@@ -13705,15 +13652,13 @@
       <c r="D192" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E192" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E192" s="7"/>
       <c r="F192" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G192" s="7" t="str">
+      <c r="G192" s="7" t="e">
         <f>+VLOOKUP(E192,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H192" s="8">
         <v>46174</v>
@@ -13731,7 +13676,7 @@
         <v>828822.7</v>
       </c>
     </row>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" s="6" t="s">
         <v>116</v>
       </c>
@@ -13744,9 +13689,7 @@
       <c r="D193" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E193" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E193" s="7"/>
       <c r="F193" s="6" t="s">
         <v>185</v>
       </c>
@@ -13769,7 +13712,7 @@
         <v>817483.96</v>
       </c>
     </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" s="6" t="s">
         <v>116</v>
       </c>
@@ -13782,15 +13725,13 @@
       <c r="D194" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E194" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E194" s="7"/>
       <c r="F194" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G194" s="7" t="str">
+      <c r="G194" s="7" t="e">
         <f>+VLOOKUP(E194,Detail!$E$51:$F$95,2,0)</f>
-        <v>INF179K01VK7</v>
+        <v>#N/A</v>
       </c>
       <c r="H194" s="8">
         <v>46157</v>
@@ -13808,7 +13749,7 @@
         <v>897442.94</v>
       </c>
     </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" s="6" t="s">
         <v>116</v>
       </c>
@@ -13821,9 +13762,7 @@
       <c r="D195" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E195" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E195" s="7"/>
       <c r="F195" s="6" t="s">
         <v>185</v>
       </c>
@@ -13846,7 +13785,7 @@
         <v>1432882.64</v>
       </c>
     </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" s="6" t="s">
         <v>116</v>
       </c>
@@ -13859,9 +13798,7 @@
       <c r="D196" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E196" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E196" s="7"/>
       <c r="F196" s="6" t="s">
         <v>185</v>
       </c>
@@ -13884,7 +13821,7 @@
         <v>561879.43999999994</v>
       </c>
     </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" s="6" t="s">
         <v>116</v>
       </c>
@@ -13923,7 +13860,7 @@
         <v>401727.34</v>
       </c>
     </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" s="6" t="s">
         <v>116</v>
       </c>
@@ -13962,7 +13899,7 @@
         <v>463147.44</v>
       </c>
     </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" s="6" t="s">
         <v>116</v>
       </c>
@@ -14001,7 +13938,7 @@
         <v>415851.25</v>
       </c>
     </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" s="6" t="s">
         <v>116</v>
       </c>
@@ -14039,7 +13976,7 @@
         <v>507942.72</v>
       </c>
     </row>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" s="6" t="s">
         <v>116</v>
       </c>
@@ -14077,7 +14014,7 @@
         <v>978374.36</v>
       </c>
     </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" s="6" t="s">
         <v>116</v>
       </c>
@@ -14116,7 +14053,7 @@
         <v>1022850.43</v>
       </c>
     </row>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" s="6" t="s">
         <v>116</v>
       </c>
@@ -14155,7 +14092,7 @@
         <v>782689.1</v>
       </c>
     </row>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" s="6" t="s">
         <v>116</v>
       </c>
@@ -14194,7 +14131,7 @@
         <v>653041.28</v>
       </c>
     </row>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" s="6" t="s">
         <v>116</v>
       </c>
@@ -14233,7 +14170,7 @@
         <v>897314.25</v>
       </c>
     </row>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" s="6" t="s">
         <v>116</v>
       </c>
@@ -14272,7 +14209,7 @@
         <v>689096.14</v>
       </c>
     </row>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" s="6" t="s">
         <v>116</v>
       </c>
@@ -14311,7 +14248,7 @@
         <v>660304.82999999996</v>
       </c>
     </row>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" s="6" t="s">
         <v>116</v>
       </c>
@@ -14350,7 +14287,7 @@
         <v>1752990.85</v>
       </c>
     </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" s="6" t="s">
         <v>116</v>
       </c>
@@ -14389,7 +14326,7 @@
         <v>697180.52</v>
       </c>
     </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" s="6" t="s">
         <v>116</v>
       </c>
@@ -14428,7 +14365,7 @@
         <v>1203746.96</v>
       </c>
     </row>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" s="6" t="s">
         <v>116</v>
       </c>
@@ -14467,7 +14404,7 @@
         <v>900238.71</v>
       </c>
     </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" s="6" t="s">
         <v>116</v>
       </c>
@@ -14506,7 +14443,7 @@
         <v>301947.52000000002</v>
       </c>
     </row>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" s="6" t="s">
         <v>116</v>
       </c>
@@ -14545,7 +14482,7 @@
         <v>919767.09</v>
       </c>
     </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" s="6" t="s">
         <v>116</v>
       </c>
@@ -14584,7 +14521,7 @@
         <v>709690.89</v>
       </c>
     </row>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" s="6" t="s">
         <v>116</v>
       </c>
@@ -14623,7 +14560,7 @@
         <v>918272.42</v>
       </c>
     </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" s="6" t="s">
         <v>116</v>
       </c>
@@ -14662,7 +14599,7 @@
         <v>1843228.86</v>
       </c>
     </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" s="6" t="s">
         <v>116</v>
       </c>
@@ -14701,7 +14638,7 @@
         <v>933917.01</v>
       </c>
     </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" s="6" t="s">
         <v>116</v>
       </c>
@@ -14740,7 +14677,7 @@
         <v>686901.61</v>
       </c>
     </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" s="6" t="s">
         <v>116</v>
       </c>
@@ -14779,7 +14716,7 @@
         <v>17026.439999999999</v>
       </c>
     </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" s="6" t="s">
         <v>116</v>
       </c>
@@ -14818,7 +14755,7 @@
         <v>916484.42</v>
       </c>
     </row>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" s="6" t="s">
         <v>116</v>
       </c>
@@ -14857,7 +14794,7 @@
         <v>833889.42</v>
       </c>
     </row>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" s="6" t="s">
         <v>116</v>
       </c>
@@ -14896,7 +14833,7 @@
         <v>958028.24</v>
       </c>
     </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" s="6" t="s">
         <v>116</v>
       </c>
@@ -14935,7 +14872,7 @@
         <v>1125529.79</v>
       </c>
     </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" s="6" t="s">
         <v>116</v>
       </c>
@@ -14974,7 +14911,7 @@
         <v>776573.22</v>
       </c>
     </row>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" s="6" t="s">
         <v>116</v>
       </c>
@@ -15013,7 +14950,7 @@
         <v>781564.19</v>
       </c>
     </row>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" s="6" t="s">
         <v>116</v>
       </c>
@@ -15052,7 +14989,7 @@
         <v>815780.68</v>
       </c>
     </row>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" s="6" t="s">
         <v>116</v>
       </c>
@@ -15090,7 +15027,7 @@
         <v>872771.17</v>
       </c>
     </row>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" s="6" t="s">
         <v>116</v>
       </c>
@@ -15129,7 +15066,7 @@
         <v>747453.31</v>
       </c>
     </row>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" s="6" t="s">
         <v>116</v>
       </c>
@@ -15168,7 +15105,7 @@
         <v>15759.34</v>
       </c>
     </row>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" s="6" t="s">
         <v>116</v>
       </c>
@@ -15207,7 +15144,7 @@
         <v>216372.03</v>
       </c>
     </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" s="6" t="s">
         <v>116</v>
       </c>
@@ -15245,7 +15182,7 @@
         <v>330069.95</v>
       </c>
     </row>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" s="6" t="s">
         <v>116</v>
       </c>
@@ -15284,7 +15221,7 @@
         <v>404625.73</v>
       </c>
     </row>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" s="6" t="s">
         <v>116</v>
       </c>
@@ -15323,7 +15260,7 @@
         <v>340348.26</v>
       </c>
     </row>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" s="6" t="s">
         <v>116</v>
       </c>
@@ -15362,7 +15299,7 @@
         <v>471800.42</v>
       </c>
     </row>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" s="6" t="s">
         <v>116</v>
       </c>
@@ -15401,7 +15338,7 @@
         <v>391270.79</v>
       </c>
     </row>
-    <row r="236" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A236" s="6" t="s">
         <v>116</v>
       </c>
@@ -15440,7 +15377,7 @@
         <v>347712.01</v>
       </c>
     </row>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" s="6" t="s">
         <v>116</v>
       </c>
@@ -15479,7 +15416,7 @@
         <v>310260.32</v>
       </c>
     </row>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" s="6" t="s">
         <v>116</v>
       </c>
@@ -15518,7 +15455,7 @@
         <v>192136.55</v>
       </c>
     </row>
-    <row r="239" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A239" s="6" t="s">
         <v>116</v>
       </c>
@@ -15557,7 +15494,7 @@
         <v>288877.65999999997</v>
       </c>
     </row>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" s="6" t="s">
         <v>116</v>
       </c>
@@ -15596,7 +15533,7 @@
         <v>721473.28</v>
       </c>
     </row>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A241" s="6" t="s">
         <v>116</v>
       </c>
@@ -15635,7 +15572,7 @@
         <v>436847.66</v>
       </c>
     </row>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" s="6" t="s">
         <v>116</v>
       </c>
@@ -15674,7 +15611,7 @@
         <v>255430.49</v>
       </c>
     </row>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A243" s="6" t="s">
         <v>116</v>
       </c>
@@ -15713,7 +15650,7 @@
         <v>354676.47</v>
       </c>
     </row>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" s="6" t="s">
         <v>116</v>
       </c>
@@ -15752,7 +15689,7 @@
         <v>324846.27</v>
       </c>
     </row>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" s="6" t="s">
         <v>116</v>
       </c>
@@ -15791,7 +15728,7 @@
         <v>327913.93</v>
       </c>
     </row>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" s="6" t="s">
         <v>116</v>
       </c>
@@ -15830,7 +15767,7 @@
         <v>340537.64</v>
       </c>
     </row>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" s="6" t="s">
         <v>116</v>
       </c>
@@ -15869,7 +15806,7 @@
         <v>342194.51</v>
       </c>
     </row>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" s="6" t="s">
         <v>116</v>
       </c>
@@ -15908,7 +15845,7 @@
         <v>284956.15999999997</v>
       </c>
     </row>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" s="6" t="s">
         <v>116</v>
       </c>
@@ -15947,7 +15884,7 @@
         <v>599374.22</v>
       </c>
     </row>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" s="6" t="s">
         <v>116</v>
       </c>
@@ -15986,7 +15923,7 @@
         <v>387156.4</v>
       </c>
     </row>
-    <row r="251" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" s="6" t="s">
         <v>116</v>
       </c>
@@ -16025,7 +15962,7 @@
         <v>310246.12</v>
       </c>
     </row>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" s="6" t="s">
         <v>116</v>
       </c>
@@ -16063,7 +16000,7 @@
         <v>394049.3</v>
       </c>
     </row>
-    <row r="253" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" s="6" t="s">
         <v>116</v>
       </c>
@@ -16102,7 +16039,7 @@
         <v>44783.01</v>
       </c>
     </row>
-    <row r="254" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" s="6" t="s">
         <v>116</v>
       </c>
@@ -16141,7 +16078,7 @@
         <v>206797.44</v>
       </c>
     </row>
-    <row r="255" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" s="6" t="s">
         <v>116</v>
       </c>
@@ -16180,7 +16117,7 @@
         <v>180508.24</v>
       </c>
     </row>
-    <row r="256" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" s="6" t="s">
         <v>116</v>
       </c>
@@ -16219,7 +16156,7 @@
         <v>301401.21000000002</v>
       </c>
     </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A257" s="6" t="s">
         <v>116</v>
       </c>
@@ -16258,7 +16195,7 @@
         <v>31947.51</v>
       </c>
     </row>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" s="6" t="s">
         <v>116</v>
       </c>
@@ -16297,7 +16234,7 @@
         <v>55274.45</v>
       </c>
     </row>
-    <row r="259" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" s="6" t="s">
         <v>116</v>
       </c>
@@ -16336,7 +16273,7 @@
         <v>295880.96999999997</v>
       </c>
     </row>
-    <row r="260" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A260" s="6" t="s">
         <v>116</v>
       </c>
@@ -16375,7 +16312,7 @@
         <v>175318.29</v>
       </c>
     </row>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A261" s="6" t="s">
         <v>116</v>
       </c>
@@ -16414,7 +16351,7 @@
         <v>128276.62</v>
       </c>
     </row>
-    <row r="262" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A262" s="6" t="s">
         <v>116</v>
       </c>
@@ -16453,7 +16390,7 @@
         <v>146348.17000000001</v>
       </c>
     </row>
-    <row r="263" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A263" s="6" t="s">
         <v>116</v>
       </c>
@@ -16492,7 +16429,7 @@
         <v>229422.7</v>
       </c>
     </row>
-    <row r="264" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A264" s="6" t="s">
         <v>116</v>
       </c>
@@ -16531,7 +16468,7 @@
         <v>19965.13</v>
       </c>
     </row>
-    <row r="265" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" s="6" t="s">
         <v>116</v>
       </c>
@@ -16570,7 +16507,7 @@
         <v>370847.08</v>
       </c>
     </row>
-    <row r="266" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A266" s="6" t="s">
         <v>116</v>
       </c>
@@ -16609,7 +16546,7 @@
         <v>43864.28</v>
       </c>
     </row>
-    <row r="267" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A267" s="6" t="s">
         <v>116</v>
       </c>
@@ -16648,7 +16585,7 @@
         <v>16566.830000000002</v>
       </c>
     </row>
-    <row r="268" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A268" s="6" t="s">
         <v>116</v>
       </c>
@@ -16686,7 +16623,7 @@
         <v>349320.04</v>
       </c>
     </row>
-    <row r="269" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A269" s="6" t="s">
         <v>116</v>
       </c>
@@ -16725,7 +16662,7 @@
         <v>811998.37</v>
       </c>
     </row>
-    <row r="270" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A270" s="6" t="s">
         <v>116</v>
       </c>
@@ -16764,7 +16701,7 @@
         <v>207126.64</v>
       </c>
     </row>
-    <row r="271" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A271" s="6" t="s">
         <v>116</v>
       </c>
@@ -16803,7 +16740,7 @@
         <v>625442.98</v>
       </c>
     </row>
-    <row r="272" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" s="6" t="s">
         <v>116</v>
       </c>
@@ -16842,7 +16779,7 @@
         <v>224242.16</v>
       </c>
     </row>
-    <row r="273" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A273" s="6" t="s">
         <v>116</v>
       </c>
@@ -16881,7 +16818,7 @@
         <v>188498.05</v>
       </c>
     </row>
-    <row r="274" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A274" s="6" t="s">
         <v>116</v>
       </c>
@@ -16920,7 +16857,7 @@
         <v>242462.72</v>
       </c>
     </row>
-    <row r="275" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A275" s="6" t="s">
         <v>116</v>
       </c>
@@ -16959,7 +16896,7 @@
         <v>246441.43</v>
       </c>
     </row>
-    <row r="276" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A276" s="6" t="s">
         <v>116</v>
       </c>
@@ -16998,7 +16935,7 @@
         <v>720603.79</v>
       </c>
     </row>
-    <row r="277" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A277" s="6" t="s">
         <v>116</v>
       </c>
@@ -17037,7 +16974,7 @@
         <v>309236.2</v>
       </c>
     </row>
-    <row r="278" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A278" s="6" t="s">
         <v>116</v>
       </c>
@@ -17075,7 +17012,7 @@
         <v>311076.08</v>
       </c>
     </row>
-    <row r="279" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A279" s="6" t="s">
         <v>116</v>
       </c>
@@ -17114,7 +17051,7 @@
         <v>253913.3</v>
       </c>
     </row>
-    <row r="280" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A280" s="6" t="s">
         <v>116</v>
       </c>
@@ -17153,7 +17090,7 @@
         <v>333170.46000000002</v>
       </c>
     </row>
-    <row r="281" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A281" s="6" t="s">
         <v>116</v>
       </c>
@@ -17192,7 +17129,7 @@
         <v>57091.01</v>
       </c>
     </row>
-    <row r="282" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A282" s="6" t="s">
         <v>116</v>
       </c>
@@ -17231,7 +17168,7 @@
         <v>58188.55</v>
       </c>
     </row>
-    <row r="283" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A283" s="6" t="s">
         <v>116</v>
       </c>
@@ -17270,7 +17207,7 @@
         <v>35056.230000000003</v>
       </c>
     </row>
-    <row r="284" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A284" s="6" t="s">
         <v>116</v>
       </c>
@@ -17309,7 +17246,7 @@
         <v>203233.06</v>
       </c>
     </row>
-    <row r="285" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A285" s="6" t="s">
         <v>116</v>
       </c>
@@ -17348,7 +17285,7 @@
         <v>238437.05</v>
       </c>
     </row>
-    <row r="286" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A286" s="6" t="s">
         <v>116</v>
       </c>
@@ -17387,7 +17324,7 @@
         <v>307296.28999999998</v>
       </c>
     </row>
-    <row r="287" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A287" s="6" t="s">
         <v>116</v>
       </c>
@@ -17425,7 +17362,7 @@
         <v>351073.6</v>
       </c>
     </row>
-    <row r="288" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A288" s="6" t="s">
         <v>116</v>
       </c>
@@ -17464,7 +17401,7 @@
         <v>439639.64</v>
       </c>
     </row>
-    <row r="289" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A289" s="6" t="s">
         <v>116</v>
       </c>
@@ -17503,7 +17440,7 @@
         <v>37692.85</v>
       </c>
     </row>
-    <row r="290" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A290" s="6" t="s">
         <v>116</v>
       </c>
@@ -17542,7 +17479,7 @@
         <v>12046.89</v>
       </c>
     </row>
-    <row r="291" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A291" s="6" t="s">
         <v>116</v>
       </c>
@@ -17581,7 +17518,7 @@
         <v>50194.79</v>
       </c>
     </row>
-    <row r="292" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A292" s="6" t="s">
         <v>116</v>
       </c>
@@ -17620,7 +17557,7 @@
         <v>35745.21</v>
       </c>
     </row>
-    <row r="293" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A293" s="6" t="s">
         <v>116</v>
       </c>
@@ -17659,7 +17596,7 @@
         <v>18843.14</v>
       </c>
     </row>
-    <row r="294" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A294" s="6" t="s">
         <v>116</v>
       </c>
@@ -17698,7 +17635,7 @@
         <v>6670.09</v>
       </c>
     </row>
-    <row r="295" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A295" s="6" t="s">
         <v>116</v>
       </c>
@@ -17737,7 +17674,7 @@
         <v>24176.63</v>
       </c>
     </row>
-    <row r="296" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A296" s="6" t="s">
         <v>116</v>
       </c>
@@ -17776,7 +17713,7 @@
         <v>47591.85</v>
       </c>
     </row>
-    <row r="297" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A297" s="6" t="s">
         <v>116</v>
       </c>
@@ -17815,7 +17752,7 @@
         <v>51913.38</v>
       </c>
     </row>
-    <row r="298" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A298" s="6" t="s">
         <v>116</v>
       </c>
@@ -17853,7 +17790,7 @@
         <v>91073.01</v>
       </c>
     </row>
-    <row r="299" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A299" s="6" t="s">
         <v>116</v>
       </c>
@@ -17892,7 +17829,7 @@
         <v>71439.42</v>
       </c>
     </row>
-    <row r="300" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A300" s="6" t="s">
         <v>116</v>
       </c>
@@ -17930,7 +17867,7 @@
         <v>40274.620000000003</v>
       </c>
     </row>
-    <row r="301" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A301" s="6" t="s">
         <v>116</v>
       </c>
@@ -17969,7 +17906,7 @@
         <v>13769.09</v>
       </c>
     </row>
-    <row r="302" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A302" s="6" t="s">
         <v>116</v>
       </c>
@@ -18007,7 +17944,7 @@
         <v>222829.67</v>
       </c>
     </row>
-    <row r="303" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A303" s="6" t="s">
         <v>116</v>
       </c>
@@ -18046,7 +17983,7 @@
         <v>51227.02</v>
       </c>
     </row>
-    <row r="304" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A304" s="6" t="s">
         <v>116</v>
       </c>
@@ -18084,7 +18021,7 @@
         <v>296506.03999999998</v>
       </c>
     </row>
-    <row r="305" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A305" s="6" t="s">
         <v>116</v>
       </c>
@@ -18123,7 +18060,7 @@
         <v>101896.82</v>
       </c>
     </row>
-    <row r="306" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A306" s="6" t="s">
         <v>116</v>
       </c>
@@ -18162,7 +18099,7 @@
         <v>96664.71</v>
       </c>
     </row>
-    <row r="307" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" s="6" t="s">
         <v>116</v>
       </c>
@@ -18201,7 +18138,7 @@
         <v>78578.61</v>
       </c>
     </row>
-    <row r="308" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A308" s="6" t="s">
         <v>116</v>
       </c>
@@ -18240,7 +18177,7 @@
         <v>354585.43</v>
       </c>
     </row>
-    <row r="309" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" s="6" t="s">
         <v>116</v>
       </c>
@@ -18278,7 +18215,7 @@
         <v>58435.58</v>
       </c>
     </row>
-    <row r="310" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" s="6" t="s">
         <v>116</v>
       </c>
@@ -18317,7 +18254,7 @@
         <v>275214.59999999998</v>
       </c>
     </row>
-    <row r="311" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A311" s="6" t="s">
         <v>116</v>
       </c>
@@ -18356,7 +18293,7 @@
         <v>23804.09</v>
       </c>
     </row>
-    <row r="312" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A312" s="6" t="s">
         <v>116</v>
       </c>
@@ -18395,7 +18332,7 @@
         <v>515652.47</v>
       </c>
     </row>
-    <row r="313" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A313" s="6" t="s">
         <v>116</v>
       </c>
@@ -18433,7 +18370,7 @@
         <v>23336.18</v>
       </c>
     </row>
-    <row r="314" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A314" s="6" t="s">
         <v>116</v>
       </c>
@@ -18472,7 +18409,7 @@
         <v>369734.37</v>
       </c>
     </row>
-    <row r="315" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A315" s="6" t="s">
         <v>116</v>
       </c>
@@ -18511,7 +18448,7 @@
         <v>269913</v>
       </c>
     </row>
-    <row r="316" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A316" s="6" t="s">
         <v>116</v>
       </c>
@@ -18550,7 +18487,7 @@
         <v>710673.83</v>
       </c>
     </row>
-    <row r="317" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A317" s="6" t="s">
         <v>116</v>
       </c>
@@ -18589,7 +18526,7 @@
         <v>546912.29</v>
       </c>
     </row>
-    <row r="318" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A318" s="6" t="s">
         <v>116</v>
       </c>
@@ -18628,7 +18565,7 @@
         <v>368991.34</v>
       </c>
     </row>
-    <row r="319" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A319" s="6" t="s">
         <v>116</v>
       </c>
@@ -18666,7 +18603,7 @@
         <v>265734.44</v>
       </c>
     </row>
-    <row r="320" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A320" s="6" t="s">
         <v>116</v>
       </c>
@@ -18705,7 +18642,7 @@
         <v>363401.91</v>
       </c>
     </row>
-    <row r="321" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A321" s="6" t="s">
         <v>116</v>
       </c>
@@ -18744,7 +18681,7 @@
         <v>272973.24</v>
       </c>
     </row>
-    <row r="322" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A322" s="6" t="s">
         <v>116</v>
       </c>
@@ -18782,7 +18719,7 @@
         <v>385188.02</v>
       </c>
     </row>
-    <row r="323" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A323" s="6" t="s">
         <v>116</v>
       </c>
@@ -18821,7 +18758,7 @@
         <v>266402.7</v>
       </c>
     </row>
-    <row r="324" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A324" s="6" t="s">
         <v>116</v>
       </c>
@@ -18860,7 +18797,7 @@
         <v>268415.82</v>
       </c>
     </row>
-    <row r="325" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A325" s="6" t="s">
         <v>116</v>
       </c>
@@ -18899,7 +18836,7 @@
         <v>358853.74</v>
       </c>
     </row>
-    <row r="326" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A326" s="6" t="s">
         <v>116</v>
       </c>
@@ -18938,7 +18875,7 @@
         <v>295401.95</v>
       </c>
     </row>
-    <row r="327" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A327" s="6" t="s">
         <v>116</v>
       </c>
@@ -18977,7 +18914,7 @@
         <v>261970.95</v>
       </c>
     </row>
-    <row r="328" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A328" s="6" t="s">
         <v>116</v>
       </c>
@@ -19016,7 +18953,7 @@
         <v>355527.97</v>
       </c>
     </row>
-    <row r="329" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A329" s="6" t="s">
         <v>116</v>
       </c>
@@ -19055,7 +18992,7 @@
         <v>534050.49</v>
       </c>
     </row>
-    <row r="330" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A330" s="6" t="s">
         <v>116</v>
       </c>
@@ -19094,7 +19031,7 @@
         <v>362837.51</v>
       </c>
     </row>
-    <row r="331" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A331" s="6" t="s">
         <v>116</v>
       </c>
@@ -19132,7 +19069,7 @@
         <v>347088</v>
       </c>
     </row>
-    <row r="332" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A332" s="6" t="s">
         <v>116</v>
       </c>
@@ -19171,7 +19108,7 @@
         <v>266399.38</v>
       </c>
     </row>
-    <row r="333" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A333" s="6" t="s">
         <v>116</v>
       </c>
@@ -19210,7 +19147,7 @@
         <v>349405.62</v>
       </c>
     </row>
-    <row r="334" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A334" s="6" t="s">
         <v>116</v>
       </c>
@@ -19249,7 +19186,7 @@
         <v>307252.21999999997</v>
       </c>
     </row>
-    <row r="335" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A335" s="6" t="s">
         <v>116</v>
       </c>
@@ -19288,7 +19225,7 @@
         <v>371173.98</v>
       </c>
     </row>
-    <row r="336" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A336" s="6" t="s">
         <v>116</v>
       </c>
@@ -19327,7 +19264,7 @@
         <v>270664.68</v>
       </c>
     </row>
-    <row r="337" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A337" s="6" t="s">
         <v>116</v>
       </c>
@@ -19366,7 +19303,7 @@
         <v>299527.14</v>
       </c>
     </row>
-    <row r="338" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A338" s="6" t="s">
         <v>116</v>
       </c>
@@ -19405,7 +19342,7 @@
         <v>268816.93</v>
       </c>
     </row>
-    <row r="339" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A339" s="6" t="s">
         <v>116</v>
       </c>
@@ -19444,7 +19381,7 @@
         <v>265952.18</v>
       </c>
     </row>
-    <row r="340" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A340" s="6" t="s">
         <v>116</v>
       </c>
@@ -19483,7 +19420,7 @@
         <v>298996.44</v>
       </c>
     </row>
-    <row r="341" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A341" s="6" t="s">
         <v>116</v>
       </c>
@@ -19522,7 +19459,7 @@
         <v>297233.84999999998</v>
       </c>
     </row>
-    <row r="342" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A342" s="6" t="s">
         <v>116</v>
       </c>
@@ -19560,7 +19497,7 @@
         <v>470926.09</v>
       </c>
     </row>
-    <row r="343" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A343" s="6" t="s">
         <v>116</v>
       </c>
@@ -19598,7 +19535,7 @@
         <v>483231</v>
       </c>
     </row>
-    <row r="344" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A344" s="6" t="s">
         <v>116</v>
       </c>
@@ -19636,7 +19573,7 @@
         <v>477313.2</v>
       </c>
     </row>
-    <row r="345" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A345" s="6" t="s">
         <v>116</v>
       </c>
@@ -19674,7 +19611,7 @@
         <v>78915.33</v>
       </c>
     </row>
-    <row r="346" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A346" s="6" t="s">
         <v>116</v>
       </c>
@@ -19712,7 +19649,7 @@
         <v>529411.29</v>
       </c>
     </row>
-    <row r="347" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A347" s="6" t="s">
         <v>116</v>
       </c>
@@ -19750,7 +19687,7 @@
         <v>399334.14</v>
       </c>
     </row>
-    <row r="348" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A348" s="6" t="s">
         <v>116</v>
       </c>
@@ -19788,7 +19725,7 @@
         <v>135993.4</v>
       </c>
     </row>
-    <row r="349" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A349" s="6" t="s">
         <v>116</v>
       </c>
@@ -19826,7 +19763,7 @@
         <v>158788.19</v>
       </c>
     </row>
-    <row r="350" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A350" s="6" t="s">
         <v>116</v>
       </c>
@@ -19864,7 +19801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="351" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A351" s="6" t="s">
         <v>116</v>
       </c>
@@ -19902,7 +19839,7 @@
         <v>125353.02</v>
       </c>
     </row>
-    <row r="352" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A352" s="6" t="s">
         <v>116</v>
       </c>
@@ -19940,7 +19877,7 @@
         <v>196169</v>
       </c>
     </row>
-    <row r="353" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A353" s="6" t="s">
         <v>116</v>
       </c>
@@ -19978,7 +19915,7 @@
         <v>62809</v>
       </c>
     </row>
-    <row r="354" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A354" s="6" t="s">
         <v>116</v>
       </c>
@@ -20016,7 +19953,7 @@
         <v>107179</v>
       </c>
     </row>
-    <row r="355" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A355" s="6" t="s">
         <v>116</v>
       </c>
@@ -20054,7 +19991,7 @@
         <v>43054</v>
       </c>
     </row>
-    <row r="356" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A356" s="6" t="s">
         <v>116</v>
       </c>
@@ -20092,7 +20029,7 @@
         <v>322258.96999999997</v>
       </c>
     </row>
-    <row r="357" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A357" s="6" t="s">
         <v>116</v>
       </c>
@@ -20130,7 +20067,7 @@
         <v>107632.8</v>
       </c>
     </row>
-    <row r="358" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A358" s="6" t="s">
         <v>116</v>
       </c>
@@ -20168,7 +20105,7 @@
         <v>214128.14</v>
       </c>
     </row>
-    <row r="359" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A359" s="6" t="s">
         <v>116</v>
       </c>
@@ -20206,7 +20143,7 @@
         <v>269025.81</v>
       </c>
     </row>
-    <row r="360" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A360" s="6" t="s">
         <v>116</v>
       </c>
@@ -20244,7 +20181,7 @@
         <v>79797.25</v>
       </c>
     </row>
-    <row r="361" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A361" s="6" t="s">
         <v>116</v>
       </c>
@@ -20282,7 +20219,7 @@
         <v>288790.95</v>
       </c>
     </row>
-    <row r="362" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A362" s="6" t="s">
         <v>116</v>
       </c>
@@ -20320,7 +20257,7 @@
         <v>178460.94</v>
       </c>
     </row>
-    <row r="363" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A363" s="6" t="s">
         <v>116</v>
       </c>
@@ -20358,7 +20295,7 @@
         <v>63930.080000000002</v>
       </c>
     </row>
-    <row r="364" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A364" s="6" t="s">
         <v>116</v>
       </c>
@@ -20396,7 +20333,7 @@
         <v>213765.2</v>
       </c>
     </row>
-    <row r="365" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A365" s="6" t="s">
         <v>116</v>
       </c>
@@ -20434,7 +20371,7 @@
         <v>105379.68</v>
       </c>
     </row>
-    <row r="366" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A366" s="6" t="s">
         <v>116</v>
       </c>
@@ -20472,7 +20409,7 @@
         <v>397878.63</v>
       </c>
     </row>
-    <row r="367" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A367" s="6" t="s">
         <v>116</v>
       </c>
@@ -20510,7 +20447,7 @@
         <v>49791.76</v>
       </c>
     </row>
-    <row r="368" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A368" s="6" t="s">
         <v>116</v>
       </c>
@@ -20548,7 +20485,7 @@
         <v>2504849.0099999998</v>
       </c>
     </row>
-    <row r="369" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A369" s="6" t="s">
         <v>116</v>
       </c>
@@ -20586,7 +20523,7 @@
         <v>254587.27</v>
       </c>
     </row>
-    <row r="370" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A370" s="6" t="s">
         <v>116</v>
       </c>
@@ -20624,7 +20561,7 @@
         <v>212955.17</v>
       </c>
     </row>
-    <row r="371" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A371" s="6" t="s">
         <v>116</v>
       </c>
@@ -20662,7 +20599,7 @@
         <v>130095.47</v>
       </c>
     </row>
-    <row r="372" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A372" s="6" t="s">
         <v>116</v>
       </c>
@@ -20700,7 +20637,7 @@
         <v>130117</v>
       </c>
     </row>
-    <row r="373" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A373" s="6" t="s">
         <v>116</v>
       </c>
@@ -20738,7 +20675,7 @@
         <v>451986.66</v>
       </c>
     </row>
-    <row r="374" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A374" s="6" t="s">
         <v>116</v>
       </c>
@@ -20776,7 +20713,7 @@
         <v>438523.35</v>
       </c>
     </row>
-    <row r="375" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A375" s="6" t="s">
         <v>116</v>
       </c>
@@ -20814,7 +20751,7 @@
         <v>139670.46</v>
       </c>
     </row>
-    <row r="376" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A376" s="6" t="s">
         <v>116</v>
       </c>
@@ -20852,7 +20789,7 @@
         <v>227826.71</v>
       </c>
     </row>
-    <row r="377" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A377" s="6" t="s">
         <v>116</v>
       </c>
@@ -20890,7 +20827,7 @@
         <v>349591.03999999998</v>
       </c>
     </row>
-    <row r="378" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A378" s="6" t="s">
         <v>116</v>
       </c>
@@ -20928,7 +20865,7 @@
         <v>256565.99</v>
       </c>
     </row>
-    <row r="379" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A379" s="6" t="s">
         <v>116</v>
       </c>
@@ -20966,7 +20903,7 @@
         <v>348190</v>
       </c>
     </row>
-    <row r="380" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A380" s="6" t="s">
         <v>116</v>
       </c>
@@ -21004,7 +20941,7 @@
         <v>323635.34999999998</v>
       </c>
     </row>
-    <row r="381" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A381" s="6" t="s">
         <v>116</v>
       </c>
@@ -21042,7 +20979,7 @@
         <v>107108.15</v>
       </c>
     </row>
-    <row r="382" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A382" s="6" t="s">
         <v>116</v>
       </c>
@@ -21080,7 +21017,7 @@
         <v>214148.03</v>
       </c>
     </row>
-    <row r="383" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A383" s="6" t="s">
         <v>116</v>
       </c>
@@ -21118,7 +21055,7 @@
         <v>403067.7</v>
       </c>
     </row>
-    <row r="384" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A384" s="6" t="s">
         <v>116</v>
       </c>
@@ -21156,7 +21093,7 @@
         <v>132657.59</v>
       </c>
     </row>
-    <row r="385" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A385" s="6" t="s">
         <v>116</v>
       </c>
@@ -21192,7 +21129,7 @@
         <v>10000000</v>
       </c>
     </row>
-    <row r="386" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A386" s="6" t="s">
         <v>116</v>
       </c>
@@ -21228,7 +21165,7 @@
         <v>42500000</v>
       </c>
     </row>
-    <row r="387" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A387" s="6" t="s">
         <v>116</v>
       </c>
@@ -21264,7 +21201,7 @@
         <v>3000000</v>
       </c>
     </row>
-    <row r="388" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A388" s="6" t="s">
         <v>116</v>
       </c>
@@ -21300,7 +21237,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="389" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A389" s="6" t="s">
         <v>116</v>
       </c>
@@ -21336,7 +21273,7 @@
         <v>1518322.8</v>
       </c>
     </row>
-    <row r="390" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A390" s="6" t="s">
         <v>116</v>
       </c>
@@ -21372,7 +21309,7 @@
         <v>1518322.8</v>
       </c>
     </row>
-    <row r="391" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A391" s="6" t="s">
         <v>116</v>
       </c>
@@ -21408,7 +21345,7 @@
         <v>700100.37</v>
       </c>
     </row>
-    <row r="392" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A392" s="6" t="s">
         <v>116</v>
       </c>
@@ -21444,7 +21381,7 @@
         <v>700100.37</v>
       </c>
     </row>
-    <row r="393" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A393" s="6" t="s">
         <v>116</v>
       </c>
@@ -21480,7 +21417,7 @@
         <v>1250000</v>
       </c>
     </row>
-    <row r="394" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A394" s="6" t="s">
         <v>116</v>
       </c>
@@ -21516,7 +21453,7 @@
         <v>1250000</v>
       </c>
     </row>
-    <row r="395" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A395" s="6" t="s">
         <v>116</v>
       </c>
@@ -21552,7 +21489,7 @@
         <v>850000</v>
       </c>
     </row>
-    <row r="396" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A396" s="6" t="s">
         <v>116</v>
       </c>
@@ -21588,7 +21525,7 @@
         <v>850000</v>
       </c>
     </row>
-    <row r="397" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A397" s="6" t="s">
         <v>116</v>
       </c>
@@ -21624,7 +21561,7 @@
         <v>661266.15</v>
       </c>
     </row>
-    <row r="398" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A398" s="6" t="s">
         <v>116</v>
       </c>
@@ -21660,7 +21597,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="399" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A399" s="6" t="s">
         <v>116</v>
       </c>
@@ -21696,7 +21633,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="400" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A400" s="6" t="s">
         <v>116</v>
       </c>
@@ -21732,7 +21669,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="401" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A401" s="6" t="s">
         <v>116</v>
       </c>
@@ -21768,7 +21705,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="402" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A402" s="6" t="s">
         <v>116</v>
       </c>
@@ -21804,7 +21741,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="403" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A403" s="6" t="s">
         <v>116</v>
       </c>
@@ -21840,7 +21777,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="404" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A404" s="6" t="s">
         <v>116</v>
       </c>
@@ -21876,7 +21813,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="405" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A405" s="6" t="s">
         <v>116</v>
       </c>
@@ -21912,7 +21849,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="406" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A406" s="6" t="s">
         <v>116</v>
       </c>
@@ -21948,7 +21885,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="407" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A407" s="6" t="s">
         <v>116</v>
       </c>
@@ -21984,7 +21921,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="408" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="408" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A408" s="6" t="s">
         <v>116</v>
       </c>
@@ -22020,7 +21957,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="409" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A409" s="6" t="s">
         <v>116</v>
       </c>
@@ -22056,7 +21993,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="410" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A410" s="6" t="s">
         <v>116</v>
       </c>
@@ -22092,7 +22029,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="411" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A411" s="6" t="s">
         <v>116</v>
       </c>
@@ -22128,7 +22065,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="412" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A412" s="6" t="s">
         <v>116</v>
       </c>
@@ -22164,7 +22101,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="413" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A413" s="6" t="s">
         <v>116</v>
       </c>
@@ -22200,7 +22137,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="414" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A414" s="6" t="s">
         <v>116</v>
       </c>
@@ -22236,7 +22173,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="415" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A415" s="6" t="s">
         <v>116</v>
       </c>
@@ -22272,7 +22209,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="416" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A416" s="6" t="s">
         <v>116</v>
       </c>
@@ -22308,7 +22245,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="417" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A417" s="6" t="s">
         <v>116</v>
       </c>
@@ -22344,7 +22281,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="418" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A418" s="6" t="s">
         <v>116</v>
       </c>
@@ -22380,7 +22317,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="419" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A419" s="6" t="s">
         <v>116</v>
       </c>
@@ -22416,7 +22353,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="420" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A420" s="6" t="s">
         <v>116</v>
       </c>
@@ -22452,7 +22389,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="421" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A421" s="6" t="s">
         <v>116</v>
       </c>
@@ -22488,7 +22425,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="422" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A422" s="6" t="s">
         <v>116</v>
       </c>
@@ -22524,7 +22461,7 @@
         <v>4800000</v>
       </c>
     </row>
-    <row r="423" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A423" s="6" t="s">
         <v>116</v>
       </c>
@@ -22560,7 +22497,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="424" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="424" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A424" s="6" t="s">
         <v>116</v>
       </c>
@@ -22596,7 +22533,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="425" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="425" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A425" s="6" t="s">
         <v>116</v>
       </c>
@@ -22632,7 +22569,7 @@
         <v>7500000</v>
       </c>
     </row>
-    <row r="426" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="426" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A426" s="6" t="s">
         <v>116</v>
       </c>
@@ -22668,7 +22605,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="427" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="427" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A427" s="6" t="s">
         <v>116</v>
       </c>
@@ -22704,7 +22641,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="428" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="428" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A428" s="6" t="s">
         <v>116</v>
       </c>
@@ -22740,7 +22677,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="429" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="429" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A429" s="6" t="s">
         <v>116</v>
       </c>
@@ -22776,7 +22713,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="430" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="430" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A430" s="6" t="s">
         <v>116</v>
       </c>
@@ -22812,7 +22749,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="431" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="431" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A431" s="6" t="s">
         <v>116</v>
       </c>
@@ -22848,7 +22785,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="432" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="432" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A432" s="6" t="s">
         <v>116</v>
       </c>
@@ -22884,7 +22821,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="433" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="433" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A433" s="6" t="s">
         <v>116</v>
       </c>
@@ -22920,7 +22857,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="434" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="434" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A434" s="6" t="s">
         <v>116</v>
       </c>
@@ -22956,7 +22893,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="435" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A435" s="6" t="s">
         <v>116</v>
       </c>
@@ -22992,7 +22929,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="436" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="436" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A436" s="6" t="s">
         <v>116</v>
       </c>
@@ -23028,7 +22965,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="437" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="437" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A437" s="6" t="s">
         <v>116</v>
       </c>
@@ -23064,7 +23001,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="438" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="438" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A438" s="6" t="s">
         <v>116</v>
       </c>
@@ -23100,7 +23037,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="439" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="439" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A439" s="6" t="s">
         <v>116</v>
       </c>
@@ -23136,7 +23073,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="440" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="440" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A440" s="6" t="s">
         <v>116</v>
       </c>
@@ -23172,7 +23109,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="441" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="441" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A441" s="6" t="s">
         <v>116</v>
       </c>
@@ -23208,7 +23145,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="442" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="442" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A442" s="6" t="s">
         <v>116</v>
       </c>
@@ -23244,7 +23181,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="443" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="443" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A443" s="6" t="s">
         <v>116</v>
       </c>
@@ -23280,7 +23217,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="444" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="444" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A444" s="6" t="s">
         <v>116</v>
       </c>
@@ -23316,7 +23253,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="445" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="445" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A445" s="6" t="s">
         <v>116</v>
       </c>
@@ -23352,7 +23289,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="446" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="446" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A446" s="6" t="s">
         <v>116</v>
       </c>
@@ -23388,7 +23325,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="447" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="447" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A447" s="6" t="s">
         <v>116</v>
       </c>
@@ -23424,7 +23361,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="448" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="448" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A448" s="6" t="s">
         <v>116</v>
       </c>
@@ -23460,7 +23397,7 @@
         <v>12000000</v>
       </c>
     </row>
-    <row r="449" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="449" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A449" s="6" t="s">
         <v>116</v>
       </c>
@@ -23496,7 +23433,7 @@
         <v>565000</v>
       </c>
     </row>
-    <row r="450" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="450" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A450" s="6" t="s">
         <v>116</v>
       </c>
@@ -23532,7 +23469,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="451" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="451" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A451" s="6" t="s">
         <v>116</v>
       </c>
@@ -23568,7 +23505,7 @@
         <v>565000</v>
       </c>
     </row>
-    <row r="452" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="452" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A452" s="6" t="s">
         <v>116</v>
       </c>
@@ -23604,7 +23541,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="453" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="453" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A453" s="6" t="s">
         <v>116</v>
       </c>
@@ -23640,7 +23577,7 @@
         <v>565000</v>
       </c>
     </row>
-    <row r="454" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="454" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A454" s="6" t="s">
         <v>116</v>
       </c>
@@ -23676,7 +23613,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="455" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="455" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A455" s="6" t="s">
         <v>116</v>
       </c>
@@ -23712,7 +23649,7 @@
         <v>565000</v>
       </c>
     </row>
-    <row r="456" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="456" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A456" s="6" t="s">
         <v>116</v>
       </c>
@@ -23748,7 +23685,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="457" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="457" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A457" s="6" t="s">
         <v>116</v>
       </c>
@@ -23784,7 +23721,7 @@
         <v>565000</v>
       </c>
     </row>
-    <row r="458" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="458" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A458" s="6" t="s">
         <v>116</v>
       </c>
@@ -23820,7 +23757,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="459" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="459" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A459" s="6" t="s">
         <v>116</v>
       </c>
@@ -23856,7 +23793,7 @@
         <v>565000</v>
       </c>
     </row>
-    <row r="460" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="460" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A460" s="6" t="s">
         <v>116</v>
       </c>
@@ -23892,7 +23829,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="461" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="461" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A461" s="6" t="s">
         <v>116</v>
       </c>
@@ -23928,7 +23865,7 @@
         <v>5800000</v>
       </c>
     </row>
-    <row r="462" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="462" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A462" s="6" t="s">
         <v>116</v>
       </c>
@@ -23964,7 +23901,7 @@
         <v>5300817.8600000003</v>
       </c>
     </row>
-    <row r="463" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="463" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A463" s="6" t="s">
         <v>116</v>
       </c>
@@ -24000,7 +23937,7 @@
         <v>8004264.54</v>
       </c>
     </row>
-    <row r="464" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="464" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A464" s="6" t="s">
         <v>116</v>
       </c>
@@ -24036,7 +23973,7 @@
         <v>1385000</v>
       </c>
     </row>
-    <row r="465" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="465" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A465" s="6" t="s">
         <v>116</v>
       </c>
@@ -25402,7 +25339,7 @@
         <v>1600000</v>
       </c>
     </row>
-    <row r="501" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="501" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A501" s="6" t="s">
         <v>116</v>
       </c>
@@ -25438,7 +25375,7 @@
         <v>5003302.71</v>
       </c>
     </row>
-    <row r="502" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="502" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A502" s="6" t="s">
         <v>116</v>
       </c>
@@ -25474,7 +25411,7 @@
         <v>10000419.51</v>
       </c>
     </row>
-    <row r="503" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="503" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A503" s="6" t="s">
         <v>116</v>
       </c>
@@ -25510,7 +25447,7 @@
         <v>2098574.0499999998</v>
       </c>
     </row>
-    <row r="504" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="504" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A504" s="6" t="s">
         <v>116</v>
       </c>
@@ -25546,7 +25483,7 @@
         <v>10004198.34</v>
       </c>
     </row>
-    <row r="505" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="505" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A505" s="6" t="s">
         <v>116</v>
       </c>
@@ -25582,7 +25519,7 @@
         <v>10008246.23</v>
       </c>
     </row>
-    <row r="506" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="506" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A506" s="6" t="s">
         <v>116</v>
       </c>
@@ -25618,7 +25555,7 @@
         <v>4197016.84</v>
       </c>
     </row>
-    <row r="507" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="507" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A507" s="6" t="s">
         <v>116</v>
       </c>
@@ -25654,7 +25591,7 @@
         <v>2300000</v>
       </c>
     </row>
-    <row r="508" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="508" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A508" s="6" t="s">
         <v>116</v>
       </c>
@@ -25690,7 +25627,7 @@
         <v>21003975.75</v>
       </c>
     </row>
-    <row r="509" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="509" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A509" s="6" t="s">
         <v>116</v>
       </c>
@@ -25726,7 +25663,7 @@
         <v>12200000</v>
       </c>
     </row>
-    <row r="510" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="510" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A510" s="6" t="s">
         <v>116</v>
       </c>
@@ -25762,7 +25699,7 @@
         <v>50000000</v>
       </c>
     </row>
-    <row r="511" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="511" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A511" s="6" t="s">
         <v>116</v>
       </c>
@@ -25798,7 +25735,7 @@
         <v>18940453.960000001</v>
       </c>
     </row>
-    <row r="512" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="512" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A512" s="6" t="s">
         <v>116</v>
       </c>
@@ -25834,7 +25771,7 @@
         <v>18940453.960000001</v>
       </c>
     </row>
-    <row r="513" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="513" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A513" s="6" t="s">
         <v>116</v>
       </c>
@@ -25870,7 +25807,7 @@
         <v>18800000</v>
       </c>
     </row>
-    <row r="514" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="514" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A514" s="6" t="s">
         <v>116</v>
       </c>
@@ -25906,7 +25843,7 @@
         <v>18800000</v>
       </c>
     </row>
-    <row r="515" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="515" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A515" s="6" t="s">
         <v>116</v>
       </c>
@@ -25942,7 +25879,7 @@
         <v>45304493</v>
       </c>
     </row>
-    <row r="516" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="516" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A516" s="6" t="s">
         <v>116</v>
       </c>
@@ -25978,7 +25915,7 @@
         <v>8627343.5999999996</v>
       </c>
     </row>
-    <row r="517" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="517" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A517" s="7" t="s">
         <v>116</v>
       </c>
@@ -26012,7 +25949,7 @@
         <v>25000000</v>
       </c>
     </row>
-    <row r="518" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="518" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A518" s="7" t="s">
         <v>116</v>
       </c>
@@ -26046,7 +25983,7 @@
         <v>12500000</v>
       </c>
     </row>
-    <row r="519" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="519" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A519" s="7" t="s">
         <v>116</v>
       </c>
@@ -26056,11 +25993,11 @@
       <c r="C519" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="D519" s="12" t="s">
+      <c r="D519" s="11" t="s">
         <v>159</v>
       </c>
       <c r="E519" s="7"/>
-      <c r="F519" s="13" t="s">
+      <c r="F519" s="12" t="s">
         <v>188</v>
       </c>
       <c r="G519" s="7"/>
@@ -26080,11 +26017,14 @@
         <v>12500000</v>
       </c>
     </row>
-    <row r="520" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="E520" s="11"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L519" xr:uid="{10DD8D7D-9FD3-4B34-BD1A-D08D200D033F}"/>
+  <autoFilter ref="A1:L519" xr:uid="{10DD8D7D-9FD3-4B34-BD1A-D08D200D033F}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="HDFC Focused Fund - Growth Option - Direct Plan"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>